<commit_message>
noisy files with one hot encoding
</commit_message>
<xml_diff>
--- a/heart_DT.xlsx
+++ b/heart_DT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shukl\Documents\GitHub\heart\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12C30785-F043-4E45-941C-CE6CA3952F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9632757C-B464-43E7-8C77-39DD5F190B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{17EA2864-75EB-4856-BEA7-292655FA3F25}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{17EA2864-75EB-4856-BEA7-292655FA3F25}"/>
   </bookViews>
   <sheets>
     <sheet name="DT_0%_rank13" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="DT_20%_rank13" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="23">
   <si>
     <t>PREDICTED</t>
   </si>
@@ -433,6 +432,115 @@
   </si>
   <si>
     <t>with one hot encoding</t>
+  </si>
+  <si>
+    <r>
+      <t>tree_model = DecisionTreeClassifier(max_depth=depth,random_state=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF098156"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>22</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>,criterion=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>"entropy"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>,min_samples_split =</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF098156"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>        max_attributes =</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF795E26"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>len</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF257693"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>list</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>(df_test))</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF098156"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t>-1</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -709,7 +817,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -745,52 +853,46 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1119,55 +1221,56 @@
     <col min="3" max="3" width="12.88671875" customWidth="1"/>
     <col min="4" max="5" width="12.44140625" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" customWidth="1"/>
-    <col min="12" max="12" width="12.21875" customWidth="1"/>
-    <col min="13" max="13" width="13.21875" customWidth="1"/>
-    <col min="14" max="14" width="12.44140625" customWidth="1"/>
-    <col min="15" max="15" width="13.44140625" customWidth="1"/>
+    <col min="11" max="11" width="11" customWidth="1"/>
+    <col min="12" max="12" width="10.5546875" customWidth="1"/>
+    <col min="13" max="13" width="10.77734375" customWidth="1"/>
+    <col min="14" max="14" width="11.21875" customWidth="1"/>
+    <col min="15" max="15" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="18"/>
-      <c r="E1" s="17" t="s">
+      <c r="D1" s="20"/>
+      <c r="E1" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="18"/>
+      <c r="F1" s="20"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
-      <c r="L1" s="17" t="s">
+      <c r="L1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="18"/>
-      <c r="N1" s="17" t="s">
+      <c r="M1" s="20"/>
+      <c r="N1" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="18"/>
+      <c r="O1" s="20"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="20"/>
-      <c r="E2" s="19" t="s">
+      <c r="D2" s="22"/>
+      <c r="E2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="20"/>
+      <c r="F2" s="22"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="19" t="s">
+      <c r="L2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="M2" s="20"/>
-      <c r="N2" s="19" t="s">
+      <c r="M2" s="22"/>
+      <c r="N2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="O2" s="20"/>
+      <c r="O2" s="22"/>
     </row>
     <row r="3" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
@@ -1200,7 +1303,7 @@
       </c>
     </row>
     <row r="4" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="21" t="b">
+      <c r="A4" s="23" t="b">
         <v>1</v>
       </c>
       <c r="B4" s="5" t="s">
@@ -1218,7 +1321,7 @@
       <c r="F4" s="10">
         <v>0.31654700000000002</v>
       </c>
-      <c r="J4" s="21" t="b">
+      <c r="J4" s="23" t="b">
         <v>1</v>
       </c>
       <c r="K4" s="5" t="s">
@@ -1238,7 +1341,7 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="22"/>
+      <c r="A5" s="24"/>
       <c r="B5" s="8" t="s">
         <v>4</v>
       </c>
@@ -1254,7 +1357,7 @@
       <c r="F5" s="10">
         <v>0.85192699999999999</v>
       </c>
-      <c r="J5" s="22"/>
+      <c r="J5" s="24"/>
       <c r="K5" s="8" t="s">
         <v>4</v>
       </c>
@@ -1282,56 +1385,56 @@
       <c r="O6" s="11"/>
     </row>
     <row r="7" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="25">
+      <c r="B7" s="14"/>
+      <c r="C7" s="15">
         <v>0.83367100000000005</v>
       </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="25">
+      <c r="D7" s="16"/>
+      <c r="E7" s="15">
         <v>0.85192699999999999</v>
       </c>
-      <c r="F7" s="26"/>
-      <c r="J7" s="23" t="s">
+      <c r="F7" s="16"/>
+      <c r="J7" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="K7" s="24"/>
-      <c r="L7" s="25">
+      <c r="K7" s="14"/>
+      <c r="L7" s="15">
         <v>0.80038799999999999</v>
       </c>
-      <c r="M7" s="26"/>
-      <c r="N7" s="25">
+      <c r="M7" s="16"/>
+      <c r="N7" s="15">
         <v>0.827519</v>
       </c>
-      <c r="O7" s="26"/>
+      <c r="O7" s="16"/>
     </row>
     <row r="8" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="15">
+      <c r="B8" s="18"/>
+      <c r="C8" s="25">
         <v>0.29016799999999998</v>
       </c>
-      <c r="D8" s="16"/>
-      <c r="E8" s="15">
+      <c r="D8" s="26"/>
+      <c r="E8" s="25">
         <v>0.31654700000000002</v>
       </c>
-      <c r="F8" s="16"/>
-      <c r="J8" s="13" t="s">
+      <c r="F8" s="26"/>
+      <c r="J8" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="K8" s="14"/>
-      <c r="L8" s="27">
+      <c r="K8" s="18"/>
+      <c r="L8" s="15">
         <v>0.19961200000000001</v>
       </c>
-      <c r="M8" s="28"/>
-      <c r="N8" s="27">
+      <c r="M8" s="16"/>
+      <c r="N8" s="15">
         <v>0.172481</v>
       </c>
-      <c r="O8" s="28"/>
+      <c r="O8" s="16"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="K12" s="12" t="s">
@@ -1394,17 +1497,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="N7:O7"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="N8:O8"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="J4:J5"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="E8:F8"/>
@@ -1416,6 +1508,17 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="N8:O8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -1432,51 +1535,56 @@
     <col min="4" max="4" width="11.44140625" customWidth="1"/>
     <col min="5" max="5" width="10.77734375" customWidth="1"/>
     <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="12" max="12" width="10.33203125" customWidth="1"/>
+    <col min="13" max="13" width="9.77734375" customWidth="1"/>
+    <col min="14" max="14" width="10.44140625" customWidth="1"/>
+    <col min="15" max="15" width="10" customWidth="1"/>
+    <col min="16" max="16" width="10.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="18"/>
-      <c r="E1" s="17" t="s">
+      <c r="D1" s="20"/>
+      <c r="E1" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="18"/>
+      <c r="F1" s="20"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
-      <c r="M1" s="17" t="s">
+      <c r="M1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="18"/>
-      <c r="O1" s="17" t="s">
+      <c r="N1" s="20"/>
+      <c r="O1" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="18"/>
+      <c r="P1" s="20"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="20"/>
-      <c r="E2" s="19" t="s">
+      <c r="D2" s="22"/>
+      <c r="E2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="20"/>
+      <c r="F2" s="22"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
-      <c r="M2" s="19" t="s">
+      <c r="M2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="N2" s="20"/>
-      <c r="O2" s="19" t="s">
+      <c r="N2" s="22"/>
+      <c r="O2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="P2" s="20"/>
+      <c r="P2" s="22"/>
     </row>
     <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
@@ -1509,7 +1617,7 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="b">
+      <c r="A4" s="23" t="b">
         <v>1</v>
       </c>
       <c r="B4" s="5" t="s">
@@ -1527,7 +1635,7 @@
       <c r="F4" s="7">
         <v>0.35491600000000001</v>
       </c>
-      <c r="K4" s="21" t="b">
+      <c r="K4" s="23" t="b">
         <v>1</v>
       </c>
       <c r="L4" s="5" t="s">
@@ -1547,7 +1655,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="22"/>
+      <c r="A5" s="24"/>
       <c r="B5" s="8" t="s">
         <v>4</v>
       </c>
@@ -1563,7 +1671,7 @@
       <c r="F5" s="10">
         <v>0.84584199999999998</v>
       </c>
-      <c r="K5" s="22"/>
+      <c r="K5" s="24"/>
       <c r="L5" s="8" t="s">
         <v>4</v>
       </c>
@@ -1591,56 +1699,56 @@
       <c r="P6" s="11"/>
     </row>
     <row r="7" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="25">
+      <c r="B7" s="14"/>
+      <c r="C7" s="15">
         <v>0.83772800000000003</v>
       </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="25">
+      <c r="D7" s="16"/>
+      <c r="E7" s="15">
         <v>0.84584199999999998</v>
       </c>
-      <c r="F7" s="26"/>
-      <c r="K7" s="23" t="s">
+      <c r="F7" s="16"/>
+      <c r="K7" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="L7" s="24"/>
-      <c r="M7" s="25">
+      <c r="L7" s="14"/>
+      <c r="M7" s="15">
         <v>0.75387599999999999</v>
       </c>
-      <c r="N7" s="26"/>
-      <c r="O7" s="25">
+      <c r="N7" s="16"/>
+      <c r="O7" s="15">
         <v>0.76162799999999997</v>
       </c>
-      <c r="P7" s="26"/>
+      <c r="P7" s="16"/>
     </row>
     <row r="8" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="25">
+      <c r="B8" s="18"/>
+      <c r="C8" s="15">
         <v>0.34532400000000002</v>
       </c>
-      <c r="D8" s="26"/>
-      <c r="E8" s="25">
+      <c r="D8" s="16"/>
+      <c r="E8" s="15">
         <v>0.35491600000000001</v>
       </c>
-      <c r="F8" s="26"/>
-      <c r="K8" s="13" t="s">
+      <c r="F8" s="16"/>
+      <c r="K8" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="L8" s="14"/>
-      <c r="M8" s="25">
+      <c r="L8" s="18"/>
+      <c r="M8" s="15">
         <v>0.246193</v>
       </c>
-      <c r="N8" s="26"/>
-      <c r="O8" s="25">
+      <c r="N8" s="16"/>
+      <c r="O8" s="15">
         <v>0.24365500000000001</v>
       </c>
-      <c r="P8" s="26"/>
+      <c r="P8" s="16"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
@@ -1691,17 +1799,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="O7:P7"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="O1:P1"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="K4:K5"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="E8:F8"/>
@@ -1713,6 +1810,17 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="O8:P8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -1728,51 +1836,56 @@
     <col min="3" max="3" width="10.77734375" customWidth="1"/>
     <col min="4" max="4" width="10.33203125" customWidth="1"/>
     <col min="5" max="6" width="10.77734375" customWidth="1"/>
+    <col min="12" max="12" width="11" customWidth="1"/>
+    <col min="13" max="13" width="10.33203125" customWidth="1"/>
+    <col min="14" max="14" width="10.5546875" customWidth="1"/>
+    <col min="15" max="15" width="10.6640625" customWidth="1"/>
+    <col min="16" max="16" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="18"/>
-      <c r="E1" s="17" t="s">
+      <c r="D1" s="20"/>
+      <c r="E1" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="18"/>
+      <c r="F1" s="20"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
-      <c r="M1" s="17" t="s">
+      <c r="M1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="18"/>
-      <c r="O1" s="17" t="s">
+      <c r="N1" s="20"/>
+      <c r="O1" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="18"/>
+      <c r="P1" s="20"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="20"/>
-      <c r="E2" s="19" t="s">
+      <c r="D2" s="22"/>
+      <c r="E2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="20"/>
+      <c r="F2" s="22"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
-      <c r="M2" s="19" t="s">
+      <c r="M2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="N2" s="20"/>
-      <c r="O2" s="19" t="s">
+      <c r="N2" s="22"/>
+      <c r="O2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="P2" s="20"/>
+      <c r="P2" s="22"/>
     </row>
     <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
@@ -1805,7 +1918,7 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="b">
+      <c r="A4" s="23" t="b">
         <v>1</v>
       </c>
       <c r="B4" s="5" t="s">
@@ -1823,27 +1936,27 @@
       <c r="F4" s="7">
         <v>0.37170300000000001</v>
       </c>
-      <c r="K4" s="21" t="b">
+      <c r="K4" s="23" t="b">
         <v>1</v>
       </c>
       <c r="L4" s="5" t="s">
         <v>3</v>
       </c>
       <c r="M4" s="6">
-        <v>0.61870499999999995</v>
+        <v>0.68781700000000001</v>
       </c>
       <c r="N4" s="7">
-        <v>0.381295</v>
+        <v>0.31218299999999999</v>
       </c>
       <c r="O4" s="6">
-        <v>0.62829699999999999</v>
+        <v>0.69289299999999998</v>
       </c>
       <c r="P4" s="7">
-        <v>0.37170300000000001</v>
+        <v>0.30710700000000002</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="22"/>
+      <c r="A5" s="24"/>
       <c r="B5" s="8" t="s">
         <v>4</v>
       </c>
@@ -1859,21 +1972,21 @@
       <c r="F5" s="10">
         <v>0.79107499999999997</v>
       </c>
-      <c r="K5" s="22"/>
+      <c r="K5" s="24"/>
       <c r="L5" s="8" t="s">
         <v>4</v>
       </c>
       <c r="M5" s="9">
-        <v>0.22515199999999999</v>
+        <v>0.26938000000000001</v>
       </c>
       <c r="N5" s="10">
-        <v>0.77484799999999998</v>
+        <v>0.73062000000000005</v>
       </c>
       <c r="O5" s="9">
-        <v>0.208925</v>
+        <v>0.26162800000000003</v>
       </c>
       <c r="P5" s="10">
-        <v>0.79107499999999997</v>
+        <v>0.73837200000000003</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1887,56 +2000,56 @@
       <c r="P6" s="11"/>
     </row>
     <row r="7" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="25">
+      <c r="B7" s="14"/>
+      <c r="C7" s="15">
         <v>0.77484799999999998</v>
       </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="25">
+      <c r="D7" s="16"/>
+      <c r="E7" s="15">
         <v>0.79107499999999997</v>
       </c>
-      <c r="F7" s="26"/>
-      <c r="K7" s="23" t="s">
+      <c r="F7" s="16"/>
+      <c r="K7" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="L7" s="24"/>
-      <c r="M7" s="25">
-        <v>0.77484799999999998</v>
-      </c>
-      <c r="N7" s="26"/>
-      <c r="O7" s="25">
-        <v>0.79107499999999997</v>
-      </c>
-      <c r="P7" s="26"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="15">
+        <v>0.73062000000000005</v>
+      </c>
+      <c r="N7" s="16"/>
+      <c r="O7" s="15">
+        <v>0.73837200000000003</v>
+      </c>
+      <c r="P7" s="16"/>
     </row>
     <row r="8" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="25">
+      <c r="B8" s="18"/>
+      <c r="C8" s="15">
         <v>0.381295</v>
       </c>
-      <c r="D8" s="26"/>
-      <c r="E8" s="25">
+      <c r="D8" s="16"/>
+      <c r="E8" s="15">
         <v>0.37170300000000001</v>
       </c>
-      <c r="F8" s="26"/>
-      <c r="K8" s="13" t="s">
+      <c r="F8" s="16"/>
+      <c r="K8" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="L8" s="14"/>
-      <c r="M8" s="25">
-        <v>0.381295</v>
-      </c>
-      <c r="N8" s="26"/>
-      <c r="O8" s="25">
-        <v>0.37170300000000001</v>
-      </c>
-      <c r="P8" s="26"/>
+      <c r="L8" s="18"/>
+      <c r="M8" s="15">
+        <v>0.31218299999999999</v>
+      </c>
+      <c r="N8" s="16"/>
+      <c r="O8" s="15">
+        <v>0.30710700000000002</v>
+      </c>
+      <c r="P8" s="16"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
@@ -1948,6 +2061,11 @@
         <v>13</v>
       </c>
     </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="K14" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
         <v>10</v>
@@ -1957,45 +2075,49 @@
       <c r="A16" s="12" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="K16" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="K17" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="K18" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C19" s="12"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C20" s="12"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="L20" s="12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C21" s="12"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C22" s="12"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="L22" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C23" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="O7:P7"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="O1:P1"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="K4:K5"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="E8:F8"/>
@@ -2007,6 +2129,17 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="O8:P8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>